<commit_message>
codify owner/url/yard-location conventions (rf rev 17, dc rev 7)
- owner/charterer names use the backend's existing short form, e.g. cosco
  (rf §4.14; normalize._OWNER_DISPLAY + display_owner)
- multiple urls in one [ref] cell join with ", ", never a newline
  (rf §4.15; enforced in build_workbook, both modes)
- discovery autofills the 7 yard-location columns from an existing backend
  row for the same shipbuilder, blank if new (dc §6.7)
- rebuild 2026-06-03 discovery batch under these rules; recalc clean
</commit_message>
<xml_diff>
--- a/batches/2026-06-03_discovery_since_may_2026/lng_carrier_candidate_vessels.xlsx
+++ b/batches/2026-06-03_discovery_since_may_2026/lng_carrier_candidate_vessels.xlsx
@@ -920,8 +920,7 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>https://cyprusshippingnews.com/2026/06/02/samsung-heavy-wins-five-vessel-order/
-https://indiashippingnews.com/samsung-heavy-wins-over-1-trillion-won-worth-of-orders-from-bermuda-based-company/</t>
+          <t>https://cyprusshippingnews.com/2026/06/02/samsung-heavy-wins-five-vessel-order/, https://indiashippingnews.com/samsung-heavy-wins-over-1-trillion-won-worth-of-orders-from-bermuda-based-company/</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
@@ -949,12 +948,36 @@
           <t>South Korea</t>
         </is>
       </c>
-      <c r="Z2" s="2" t="inlineStr"/>
-      <c r="AA2" s="2" t="inlineStr"/>
-      <c r="AB2" s="2" t="inlineStr"/>
-      <c r="AC2" s="2" t="inlineStr"/>
-      <c r="AD2" s="2" t="inlineStr"/>
-      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.samsungshi.com/En/Default.aspx</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>34.89804</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>128.6045</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="inlineStr">
+        <is>
+          <t>VJW3+QV Geoje-si, Gyeongsangnam-do</t>
+        </is>
+      </c>
+      <c r="AD2" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Samsung+Heavy+industries/data=!3m1!1e3!4m10!1m2!2m1!1ssamsung+heavy+industries!3m6!1s0x356ecd83691a8fb5:0xd4204e9a1bb0ef10!8m2!3d34.8969682!4d128.6046376!15sChhzYW1zdW5nIGhlYXZ5IGluZHVzdHJpZXOSAQhzaGlweWFyZOABAA!16s%2Fg%2F1tgcpry6?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="inlineStr"/>
       <c r="AH2" s="2" t="inlineStr"/>
@@ -988,8 +1011,7 @@
       </c>
       <c r="AU2" s="5" t="inlineStr">
         <is>
-          <t>https://cyprusshippingnews.com/2026/06/02/samsung-heavy-wins-five-vessel-order/
-https://www.hellenicshippingnews.com/samsung-heavy-wins-five-vessel-order/</t>
+          <t>https://cyprusshippingnews.com/2026/06/02/samsung-heavy-wins-five-vessel-order/, https://www.hellenicshippingnews.com/samsung-heavy-wins-five-vessel-order/</t>
         </is>
       </c>
       <c r="AV2" s="5" t="inlineStr">
@@ -1004,8 +1026,7 @@
       </c>
       <c r="AX2" s="5" t="inlineStr">
         <is>
-          <t>https://www.hellenicshippingnews.com/samsung-heavy-wins-five-vessel-order/
-https://lngprime.com/asia/south-koreas-samsung-heavy-to-build-one-lng-carrier-for-252-million/187561/</t>
+          <t>https://www.hellenicshippingnews.com/samsung-heavy-wins-five-vessel-order/, https://lngprime.com/asia/south-koreas-samsung-heavy-to-build-one-lng-carrier-for-252-million/187561/</t>
         </is>
       </c>
     </row>
@@ -1087,12 +1108,36 @@
           <t>South Korea</t>
         </is>
       </c>
-      <c r="Z3" s="2" t="inlineStr"/>
-      <c r="AA3" s="2" t="inlineStr"/>
-      <c r="AB3" s="2" t="inlineStr"/>
-      <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>https://www.hanwha.com/companies/hanwha-ocean.do</t>
+        </is>
+      </c>
+      <c r="AA3" s="7" t="inlineStr">
+        <is>
+          <t>34.87385</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="inlineStr">
+        <is>
+          <t>128.6966</t>
+        </is>
+      </c>
+      <c r="AC3" s="7" t="inlineStr">
+        <is>
+          <t>VMCW+V7 Geoje-si, Gyeongsangnam-do</t>
+        </is>
+      </c>
+      <c r="AD3" s="7" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE3" s="7" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Hanwha+Ocean/data=!3m1!1e3!4m10!1m2!2m1!1sHanwha+Ocean!3m6!1s0x356ecd1d7a72f7db:0x3bfe90e7d8bf93f0!8m2!3d34.8721913!4d128.6956963!15sCgxIYW53aGEgT2NlYW5aDiIMaGFud2hhIG9jZWFukgEfc2hpcGJ1aWxkaW5nX2FuZF9yZXBhaXJfY29tcGFueZoBI0NoWkRTVWhOTUc5blMwVkpRMEZuVFVSUmRYVkVTMWhuRUFF4AEA-gEECAAQLA!16s%2Fg%2F11swmd6_76?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF3" s="7" t="inlineStr">
         <is>
           <t>174000</t>
@@ -1165,7 +1210,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Jiangnan — COSCO Shipping Energy 4x LNG (Shell charter) — vessel 1/4</t>
+          <t>Jiangnan — COSCO 4x LNG (Shell charter) — vessel 1/4</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1202,7 +1247,7 @@
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>COSCO Shipping Energy Transportation</t>
+          <t>COSCO</t>
         </is>
       </c>
       <c r="T4" s="5" t="inlineStr">
@@ -1231,12 +1276,36 @@
           <t>China</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr"/>
-      <c r="AA4" s="2" t="inlineStr"/>
-      <c r="AB4" s="2" t="inlineStr"/>
-      <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="Z4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jnshipyard.com.cn/</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>31.355766</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>121.502217</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>9G32+XJ Baoshan, Shanghai, China</t>
+        </is>
+      </c>
+      <c r="AD4" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Jiangnan+Shipyard+%EF%BC%88Group%EF%BC%89+Co.,+Ltd./@31.354923,121.4990201,752m/data=!3m2!1e3!4b1!4m6!3m5!1s0x35b27324c39e47ab:0x7a74ae921f6eb2ab!8m2!3d31.354923!4d121.501595!16s%2Fg%2F11cnpghcr_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF4" s="5" t="inlineStr">
         <is>
           <t>175000</t>
@@ -1317,7 +1386,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Jiangnan — COSCO Shipping Energy 4x LNG (Shell charter) — vessel 2/4</t>
+          <t>Jiangnan — COSCO 4x LNG (Shell charter) — vessel 2/4</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1354,7 +1423,7 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>COSCO Shipping Energy Transportation</t>
+          <t>COSCO</t>
         </is>
       </c>
       <c r="T5" s="5" t="inlineStr">
@@ -1383,12 +1452,36 @@
           <t>China</t>
         </is>
       </c>
-      <c r="Z5" s="2" t="inlineStr"/>
-      <c r="AA5" s="2" t="inlineStr"/>
-      <c r="AB5" s="2" t="inlineStr"/>
-      <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="Z5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jnshipyard.com.cn/</t>
+        </is>
+      </c>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>31.355766</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>121.502217</t>
+        </is>
+      </c>
+      <c r="AC5" s="5" t="inlineStr">
+        <is>
+          <t>9G32+XJ Baoshan, Shanghai, China</t>
+        </is>
+      </c>
+      <c r="AD5" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Jiangnan+Shipyard+%EF%BC%88Group%EF%BC%89+Co.,+Ltd./@31.354923,121.4990201,752m/data=!3m2!1e3!4b1!4m6!3m5!1s0x35b27324c39e47ab:0x7a74ae921f6eb2ab!8m2!3d31.354923!4d121.501595!16s%2Fg%2F11cnpghcr_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF5" s="5" t="inlineStr">
         <is>
           <t>175000</t>
@@ -1469,7 +1562,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Jiangnan — COSCO Shipping Energy 4x LNG (Shell charter) — vessel 3/4</t>
+          <t>Jiangnan — COSCO 4x LNG (Shell charter) — vessel 3/4</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1506,7 +1599,7 @@
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>COSCO Shipping Energy Transportation</t>
+          <t>COSCO</t>
         </is>
       </c>
       <c r="T6" s="5" t="inlineStr">
@@ -1535,12 +1628,36 @@
           <t>China</t>
         </is>
       </c>
-      <c r="Z6" s="2" t="inlineStr"/>
-      <c r="AA6" s="2" t="inlineStr"/>
-      <c r="AB6" s="2" t="inlineStr"/>
-      <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="Z6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jnshipyard.com.cn/</t>
+        </is>
+      </c>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>31.355766</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>121.502217</t>
+        </is>
+      </c>
+      <c r="AC6" s="5" t="inlineStr">
+        <is>
+          <t>9G32+XJ Baoshan, Shanghai, China</t>
+        </is>
+      </c>
+      <c r="AD6" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Jiangnan+Shipyard+%EF%BC%88Group%EF%BC%89+Co.,+Ltd./@31.354923,121.4990201,752m/data=!3m2!1e3!4b1!4m6!3m5!1s0x35b27324c39e47ab:0x7a74ae921f6eb2ab!8m2!3d31.354923!4d121.501595!16s%2Fg%2F11cnpghcr_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF6" s="5" t="inlineStr">
         <is>
           <t>175000</t>
@@ -1621,7 +1738,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Jiangnan — COSCO Shipping Energy 4x LNG (Shell charter) — vessel 4/4</t>
+          <t>Jiangnan — COSCO 4x LNG (Shell charter) — vessel 4/4</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1658,7 +1775,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>COSCO Shipping Energy Transportation</t>
+          <t>COSCO</t>
         </is>
       </c>
       <c r="T7" s="5" t="inlineStr">
@@ -1687,12 +1804,36 @@
           <t>China</t>
         </is>
       </c>
-      <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="inlineStr"/>
-      <c r="AB7" s="2" t="inlineStr"/>
-      <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jnshipyard.com.cn/</t>
+        </is>
+      </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>31.355766</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>121.502217</t>
+        </is>
+      </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>9G32+XJ Baoshan, Shanghai, China</t>
+        </is>
+      </c>
+      <c r="AD7" s="5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AE7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Jiangnan+Shipyard+%EF%BC%88Group%EF%BC%89+Co.,+Ltd./@31.354923,121.4990201,752m/data=!3m2!1e3!4b1!4m6!3m5!1s0x35b27324c39e47ab:0x7a74ae921f6eb2ab!8m2!3d31.354923!4d121.501595!16s%2Fg%2F11cnpghcr_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
       <c r="AF7" s="5" t="inlineStr">
         <is>
           <t>175000</t>

</xml_diff>